<commit_message>
Party code updated temp
</commit_message>
<xml_diff>
--- a/PartyCode.xlsx
+++ b/PartyCode.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\veraj\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\po-normalization-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5651828B-558A-4F0E-942A-72578B89370F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6873D240-38EB-43AA-BE57-C2F060C95B87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{99EBD75F-AF2A-43B3-9555-8F8B52E04ADC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{99EBD75F-AF2A-43B3-9555-8F8B52E04ADC}"/>
   </bookViews>
   <sheets>
     <sheet name="ORB_PtyUPdateReport" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="890" uniqueCount="520">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="893" uniqueCount="520">
   <si>
     <t>Party Code</t>
   </si>
@@ -1690,9 +1690,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1730,7 +1730,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1836,7 +1836,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1978,7 +1978,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1986,17 +1986,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6EB0927-B5A6-4BE7-9AEA-68E6BA930412}">
-  <dimension ref="A1:E180"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E181"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="46.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="46.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2013,7 +2013,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>20</v>
       </c>
@@ -2030,7 +2030,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>24</v>
       </c>
@@ -2047,7 +2047,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>28</v>
       </c>
@@ -2064,7 +2064,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>31</v>
       </c>
@@ -2081,7 +2081,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>35</v>
       </c>
@@ -2098,7 +2098,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>39</v>
       </c>
@@ -2115,7 +2115,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>41</v>
       </c>
@@ -2132,7 +2132,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>44</v>
       </c>
@@ -2149,7 +2149,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>48</v>
       </c>
@@ -2166,7 +2166,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>51</v>
       </c>
@@ -2183,7 +2183,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>55</v>
       </c>
@@ -2200,7 +2200,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>58</v>
       </c>
@@ -2217,7 +2217,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>61</v>
       </c>
@@ -2234,7 +2234,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>65</v>
       </c>
@@ -2251,7 +2251,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>68</v>
       </c>
@@ -2268,7 +2268,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>71</v>
       </c>
@@ -2285,7 +2285,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>74</v>
       </c>
@@ -2302,7 +2302,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>77</v>
       </c>
@@ -2319,7 +2319,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>80</v>
       </c>
@@ -2336,7 +2336,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>83</v>
       </c>
@@ -2353,7 +2353,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>86</v>
       </c>
@@ -2370,7 +2370,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>89</v>
       </c>
@@ -2387,7 +2387,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>92</v>
       </c>
@@ -2404,7 +2404,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>95</v>
       </c>
@@ -2421,7 +2421,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>98</v>
       </c>
@@ -2438,7 +2438,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>101</v>
       </c>
@@ -2455,7 +2455,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>104</v>
       </c>
@@ -2472,7 +2472,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>107</v>
       </c>
@@ -2489,7 +2489,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>110</v>
       </c>
@@ -2506,7 +2506,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>113</v>
       </c>
@@ -2523,7 +2523,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>116</v>
       </c>
@@ -2540,7 +2540,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>119</v>
       </c>
@@ -2557,7 +2557,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>122</v>
       </c>
@@ -2574,7 +2574,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>125</v>
       </c>
@@ -2591,7 +2591,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
         <v>128</v>
       </c>
@@ -2608,7 +2608,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>131</v>
       </c>
@@ -2625,7 +2625,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
         <v>134</v>
       </c>
@@ -2642,7 +2642,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
         <v>137</v>
       </c>
@@ -2659,7 +2659,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>140</v>
       </c>
@@ -2676,7 +2676,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
         <v>143</v>
       </c>
@@ -2693,7 +2693,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
         <v>146</v>
       </c>
@@ -2710,7 +2710,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
         <v>149</v>
       </c>
@@ -2727,7 +2727,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
         <v>152</v>
       </c>
@@ -2744,7 +2744,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
         <v>154</v>
       </c>
@@ -2761,7 +2761,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
         <v>156</v>
       </c>
@@ -2778,7 +2778,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
         <v>159</v>
       </c>
@@ -2795,7 +2795,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
         <v>162</v>
       </c>
@@ -2812,7 +2812,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
         <v>165</v>
       </c>
@@ -2829,7 +2829,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
         <v>168</v>
       </c>
@@ -2846,7 +2846,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
         <v>170</v>
       </c>
@@ -2863,7 +2863,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
         <v>172</v>
       </c>
@@ -2880,7 +2880,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
         <v>176</v>
       </c>
@@ -2897,7 +2897,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
         <v>180</v>
       </c>
@@ -2914,7 +2914,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
         <v>183</v>
       </c>
@@ -2931,7 +2931,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
         <v>186</v>
       </c>
@@ -2948,7 +2948,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
         <v>189</v>
       </c>
@@ -2965,7 +2965,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
         <v>191</v>
       </c>
@@ -2982,7 +2982,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
         <v>193</v>
       </c>
@@ -2999,7 +2999,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
         <v>195</v>
       </c>
@@ -3016,7 +3016,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
         <v>199</v>
       </c>
@@ -3033,7 +3033,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
         <v>203</v>
       </c>
@@ -3050,7 +3050,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
         <v>206</v>
       </c>
@@ -3067,7 +3067,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
         <v>209</v>
       </c>
@@ -3084,7 +3084,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" s="1" t="s">
         <v>212</v>
       </c>
@@ -3101,7 +3101,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66" s="1" t="s">
         <v>214</v>
       </c>
@@ -3118,7 +3118,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
         <v>217</v>
       </c>
@@ -3135,7 +3135,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
         <v>219</v>
       </c>
@@ -3152,7 +3152,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69" s="1" t="s">
         <v>221</v>
       </c>
@@ -3169,7 +3169,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" s="1" t="s">
         <v>225</v>
       </c>
@@ -3186,7 +3186,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71" s="1" t="s">
         <v>228</v>
       </c>
@@ -3203,7 +3203,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72" s="1" t="s">
         <v>231</v>
       </c>
@@ -3220,7 +3220,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
         <v>233</v>
       </c>
@@ -3237,7 +3237,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
         <v>237</v>
       </c>
@@ -3254,7 +3254,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75" s="1" t="s">
         <v>240</v>
       </c>
@@ -3271,7 +3271,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
         <v>242</v>
       </c>
@@ -3288,7 +3288,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A77" s="1" t="s">
         <v>245</v>
       </c>
@@ -3305,7 +3305,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A78" s="1" t="s">
         <v>248</v>
       </c>
@@ -3322,7 +3322,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A79" s="1" t="s">
         <v>251</v>
       </c>
@@ -3339,7 +3339,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A80" s="1" t="s">
         <v>253</v>
       </c>
@@ -3356,7 +3356,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A81" s="1" t="s">
         <v>255</v>
       </c>
@@ -3373,7 +3373,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A82" s="1" t="s">
         <v>258</v>
       </c>
@@ -3390,7 +3390,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A83" s="1" t="s">
         <v>261</v>
       </c>
@@ -3407,7 +3407,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A84" s="1" t="s">
         <v>264</v>
       </c>
@@ -3424,7 +3424,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A85" s="1" t="s">
         <v>267</v>
       </c>
@@ -3441,7 +3441,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A86" s="1" t="s">
         <v>270</v>
       </c>
@@ -3458,7 +3458,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87" s="1" t="s">
         <v>273</v>
       </c>
@@ -3475,7 +3475,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A88" s="1" t="s">
         <v>275</v>
       </c>
@@ -3492,7 +3492,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A89" s="1" t="s">
         <v>277</v>
       </c>
@@ -3509,7 +3509,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A90" s="1" t="s">
         <v>279</v>
       </c>
@@ -3526,7 +3526,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A91" s="1" t="s">
         <v>282</v>
       </c>
@@ -3543,7 +3543,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A92" s="1" t="s">
         <v>288</v>
       </c>
@@ -3560,7 +3560,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A93" s="1" t="s">
         <v>291</v>
       </c>
@@ -3577,7 +3577,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A94" s="1" t="s">
         <v>294</v>
       </c>
@@ -3594,7 +3594,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A95" s="1" t="s">
         <v>297</v>
       </c>
@@ -3611,7 +3611,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A96" s="1" t="s">
         <v>299</v>
       </c>
@@ -3628,7 +3628,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A97" s="1" t="s">
         <v>302</v>
       </c>
@@ -3645,7 +3645,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A98" s="1" t="s">
         <v>305</v>
       </c>
@@ -3662,7 +3662,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A99" s="1" t="s">
         <v>308</v>
       </c>
@@ -3679,7 +3679,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A100" s="1" t="s">
         <v>311</v>
       </c>
@@ -3696,7 +3696,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A101" s="1" t="s">
         <v>313</v>
       </c>
@@ -3713,7 +3713,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A102" s="1" t="s">
         <v>315</v>
       </c>
@@ -3730,7 +3730,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A103" s="1" t="s">
         <v>317</v>
       </c>
@@ -3747,7 +3747,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A104" s="1" t="s">
         <v>319</v>
       </c>
@@ -3764,7 +3764,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A105" s="1" t="s">
         <v>322</v>
       </c>
@@ -3781,7 +3781,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A106" s="1" t="s">
         <v>325</v>
       </c>
@@ -3798,7 +3798,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A107" s="1" t="s">
         <v>328</v>
       </c>
@@ -3815,7 +3815,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A108" s="1" t="s">
         <v>331</v>
       </c>
@@ -3832,7 +3832,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A109" s="1" t="s">
         <v>334</v>
       </c>
@@ -3849,7 +3849,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A110" s="1" t="s">
         <v>338</v>
       </c>
@@ -3866,7 +3866,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A111" s="1" t="s">
         <v>341</v>
       </c>
@@ -3883,7 +3883,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A112" s="1" t="s">
         <v>344</v>
       </c>
@@ -3900,7 +3900,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A113" s="1" t="s">
         <v>346</v>
       </c>
@@ -3917,7 +3917,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A114" s="1" t="s">
         <v>348</v>
       </c>
@@ -3934,7 +3934,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A115" s="1" t="s">
         <v>350</v>
       </c>
@@ -3951,7 +3951,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A116" s="1" t="s">
         <v>353</v>
       </c>
@@ -3968,7 +3968,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A117" s="1" t="s">
         <v>356</v>
       </c>
@@ -3985,7 +3985,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A118" s="1" t="s">
         <v>358</v>
       </c>
@@ -4002,7 +4002,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A119" s="1" t="s">
         <v>361</v>
       </c>
@@ -4019,7 +4019,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A120" s="1" t="s">
         <v>363</v>
       </c>
@@ -4036,7 +4036,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A121" s="1" t="s">
         <v>366</v>
       </c>
@@ -4053,7 +4053,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A122" s="1" t="s">
         <v>368</v>
       </c>
@@ -4070,7 +4070,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A123" s="1" t="s">
         <v>371</v>
       </c>
@@ -4087,7 +4087,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A124" s="1" t="s">
         <v>374</v>
       </c>
@@ -4104,7 +4104,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A125" s="1" t="s">
         <v>378</v>
       </c>
@@ -4121,7 +4121,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A126" s="1" t="s">
         <v>381</v>
       </c>
@@ -4138,7 +4138,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A127" s="1" t="s">
         <v>383</v>
       </c>
@@ -4155,7 +4155,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A128" s="1" t="s">
         <v>385</v>
       </c>
@@ -4172,7 +4172,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A129" s="1" t="s">
         <v>387</v>
       </c>
@@ -4189,7 +4189,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A130" s="1" t="s">
         <v>389</v>
       </c>
@@ -4206,7 +4206,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A131" s="1" t="s">
         <v>392</v>
       </c>
@@ -4223,7 +4223,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A132" s="1" t="s">
         <v>395</v>
       </c>
@@ -4240,7 +4240,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A133" s="1" t="s">
         <v>397</v>
       </c>
@@ -4257,7 +4257,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A134" s="1" t="s">
         <v>399</v>
       </c>
@@ -4274,7 +4274,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A135" s="1" t="s">
         <v>401</v>
       </c>
@@ -4291,7 +4291,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A136" s="1" t="s">
         <v>403</v>
       </c>
@@ -4308,7 +4308,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A137" s="1" t="s">
         <v>406</v>
       </c>
@@ -4325,7 +4325,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A138" s="1" t="s">
         <v>408</v>
       </c>
@@ -4342,7 +4342,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A139" s="1" t="s">
         <v>411</v>
       </c>
@@ -4359,7 +4359,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A140" s="1" t="s">
         <v>413</v>
       </c>
@@ -4376,7 +4376,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A141" s="1" t="s">
         <v>416</v>
       </c>
@@ -4393,7 +4393,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A142" s="1" t="s">
         <v>418</v>
       </c>
@@ -4410,7 +4410,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A143" s="1" t="s">
         <v>420</v>
       </c>
@@ -4427,7 +4427,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A144" s="1" t="s">
         <v>423</v>
       </c>
@@ -4444,7 +4444,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A145" s="1" t="s">
         <v>426</v>
       </c>
@@ -4461,7 +4461,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A146" s="1" t="s">
         <v>429</v>
       </c>
@@ -4478,7 +4478,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A147" s="1" t="s">
         <v>431</v>
       </c>
@@ -4495,7 +4495,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A148" s="1" t="s">
         <v>434</v>
       </c>
@@ -4512,7 +4512,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A149" s="1" t="s">
         <v>436</v>
       </c>
@@ -4529,7 +4529,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A150" s="1" t="s">
         <v>438</v>
       </c>
@@ -4546,7 +4546,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A151" s="1" t="s">
         <v>441</v>
       </c>
@@ -4563,7 +4563,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A152" s="1" t="s">
         <v>443</v>
       </c>
@@ -4580,7 +4580,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A153" s="1" t="s">
         <v>446</v>
       </c>
@@ -4597,7 +4597,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A154" s="1" t="s">
         <v>448</v>
       </c>
@@ -4614,7 +4614,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A155" s="1" t="s">
         <v>450</v>
       </c>
@@ -4631,7 +4631,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A156" s="1" t="s">
         <v>453</v>
       </c>
@@ -4648,7 +4648,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A157" s="1" t="s">
         <v>455</v>
       </c>
@@ -4665,7 +4665,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A158" s="1" t="s">
         <v>458</v>
       </c>
@@ -4682,7 +4682,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A159" s="1" t="s">
         <v>460</v>
       </c>
@@ -4699,7 +4699,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A160" s="1" t="s">
         <v>463</v>
       </c>
@@ -4716,7 +4716,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A161" s="1" t="s">
         <v>465</v>
       </c>
@@ -4733,7 +4733,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A162" s="1" t="s">
         <v>468</v>
       </c>
@@ -4750,7 +4750,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A163" s="1" t="s">
         <v>471</v>
       </c>
@@ -4767,7 +4767,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A164" s="1" t="s">
         <v>473</v>
       </c>
@@ -4784,7 +4784,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A165" s="1" t="s">
         <v>418</v>
       </c>
@@ -4801,7 +4801,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A166" s="1" t="s">
         <v>477</v>
       </c>
@@ -4818,7 +4818,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A167" s="1" t="s">
         <v>480</v>
       </c>
@@ -4835,7 +4835,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A168" s="1" t="s">
         <v>482</v>
       </c>
@@ -4852,7 +4852,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A169" s="1" t="s">
         <v>484</v>
       </c>
@@ -4869,7 +4869,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A170" s="1" t="s">
         <v>486</v>
       </c>
@@ -4886,7 +4886,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A171" s="1" t="s">
         <v>489</v>
       </c>
@@ -4903,7 +4903,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A172" s="1" t="s">
         <v>491</v>
       </c>
@@ -4920,7 +4920,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A173" s="1" t="s">
         <v>494</v>
       </c>
@@ -4937,7 +4937,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A174" s="4" t="s">
         <v>513</v>
       </c>
@@ -4954,7 +4954,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A175" s="5">
         <v>336</v>
       </c>
@@ -4971,7 +4971,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A176" s="5">
         <v>5</v>
       </c>
@@ -4988,7 +4988,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A177" s="6">
         <v>337</v>
       </c>
@@ -5005,7 +5005,7 @@
         <v>122103</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A178" s="6">
         <v>338</v>
       </c>
@@ -5022,7 +5022,7 @@
         <v>140417</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A179" s="6">
         <v>340</v>
       </c>
@@ -5039,7 +5039,7 @@
         <v>501510</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A180" s="6">
         <v>339</v>
       </c>
@@ -5054,6 +5054,23 @@
       </c>
       <c r="E180" s="6">
         <v>501401</v>
+      </c>
+    </row>
+    <row r="181" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A181" s="6">
+        <v>340</v>
+      </c>
+      <c r="B181" s="1" t="s">
+        <v>512</v>
+      </c>
+      <c r="C181" s="6" t="s">
+        <v>519</v>
+      </c>
+      <c r="D181" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="E181" s="6">
+        <v>501402</v>
       </c>
     </row>
   </sheetData>

</xml_diff>